<commit_message>
Implementation sheet: make every SKOS value name a real concept
All 15 filled cells in the 'XAS skos uri' column were checked against
XAS_Glossary_SKOS.json. Twelve named no concept that exists: eight used
underscores the glossary does not (xas:facility_energy ->
xas:facilityenergy) and four differed only in case (xas:Instrument ->
xas:instrument, xas:Beamline, xas:AnalysisEvent, xas:installedOptions).
Every one had an obvious target; nothing was guessed.

Edited the shared strings in place and copied every other zip part
byte-for-byte, so the three cell comments and the VML drawing survive --
openpyxl would have rewritten the workbook and is known to drop them.
Each of the twelve strings was verified unique and used in exactly one
cell first.

The column is still empty in 47 of 62 rows.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XAS-CDIFImplementation-revised.xlsx
+++ b/XAS-CDIFImplementation-revised.xlsx
@@ -227,7 +227,7 @@
     <t>units should be joules, product of current and particle energy.</t>
   </si>
   <si>
-    <t>xas:facility_energy</t>
+    <t>xas:facilityenergy</t>
   </si>
   <si>
     <t>current</t>
@@ -244,7 +244,7 @@
     <t>Units A/mA/microA. Facility modeled as schema:location Place on the wasGeneratedBy Event (was: contributor Role).</t>
   </si>
   <si>
-    <t>xas:facility_current</t>
+    <t>xas:facilitycurrent</t>
   </si>
   <si>
     <t>x-ray source</t>
@@ -321,7 +321,7 @@
     <t>prov:wasGeneratedBy/@type:schema:Action, prov:Activity, 'xas:AnalysisEvent'</t>
   </si>
   <si>
-    <t>xas:AnalysisEvent</t>
+    <t>xas:analysisevent</t>
   </si>
   <si>
     <t>CalibrationDescription</t>
@@ -357,7 +357,7 @@
     <t>xas:installedOptions in property vocabulary. Can thes options be represented as instrument components (e.g. see all the things in the NXinstrument group in NEXUS)</t>
   </si>
   <si>
-    <t>xas:installedOptions</t>
+    <t>xas:installedoptions</t>
   </si>
   <si>
     <t>Environmental conditions</t>
@@ -392,7 +392,7 @@
    schema:additionalType + schema:additionalProperty (see rows below)</t>
   </si>
   <si>
-    <t>xas:Instrument</t>
+    <t>xas:instrument</t>
   </si>
   <si>
     <t>Instrument/name</t>
@@ -500,7 +500,7 @@
     <t>partOf xas:Instrument, IsA xas:Instrument.  How is XDI beamline related to NEXUS NXbeam?</t>
   </si>
   <si>
-    <t>xas:Beamline</t>
+    <t>xas:beamline</t>
   </si>
   <si>
     <t>Instrument/beamline/name</t>
@@ -545,7 +545,7 @@
     <t>xas:harmonic_rejection in property vocabulary</t>
   </si>
   <si>
-    <t>xas:harmonic_rejection</t>
+    <t>xas:harmonicrejection</t>
   </si>
   <si>
     <t>Instrument/monitor</t>
@@ -590,7 +590,7 @@
     <t>in the instrument section, list the various detectors used to measure incident and transmitted or fluorescent intensity/flux</t>
   </si>
   <si>
-    <t>xas:detector_type</t>
+    <t>xas:detectortype</t>
   </si>
   <si>
     <t>Instrument/detector/i0</t>
@@ -623,7 +623,7 @@
     <t>schema:variableMeasured/@type=cdi:InstanceVariable/{..."schema:propertyID": {"@id": "xas:Reference_Intensity"},schema:measurementTechnique:{"@id":"uri for detector type instance"}</t>
   </si>
   <si>
-    <t>xas:Reference_Intensity</t>
+    <t>xas:referenceintensity</t>
   </si>
   <si>
     <t>Sample</t>
@@ -666,7 +666,7 @@
                     schema:additionalType: MaterialSample, additionalProperty:{ schema:propertyID: 'xas:sample_preparation',</t>
   </si>
   <si>
-    <t>xas:sample_preparation</t>
+    <t>xas:samplepreparation</t>
   </si>
   <si>
     <t>sample/size</t>
@@ -712,7 +712,7 @@
                     schema:additionalType: MaterialSample, additionalProperty:{ schema:propertyID: 'xas:parent_sample',</t>
   </si>
   <si>
-    <t>xas:parent_sample</t>
+    <t>xas:parentsample</t>
   </si>
   <si>
     <t>sample/state</t>
@@ -725,7 +725,7 @@
     <t>Suggest using material type vocabulary like https://vocabs.ardc.edu.au/viewById/664</t>
   </si>
   <si>
-    <t>xas:sample_material</t>
+    <t>xas:samplematerial</t>
   </si>
   <si>
     <t>Scan.number</t>

</xml_diff>